<commit_message>
Count postponement capacity from the first round of each league
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019JaUXG9cM9tqcS3gAAknD4
</commit_message>
<xml_diff>
--- a/نتيجة_المباريات_المؤجلة_2026-27.xlsx
+++ b/نتيجة_المباريات_المؤجلة_2026-27.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -478,7 +478,8 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="90" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="90" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1">
@@ -514,6 +515,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>منها مواعيد ما زالت متاحة بعد اليوم 22/10/2026</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>التواريخ المقترحة للمباريات المؤجلة</t>
         </is>
       </c>
@@ -540,14 +546,17 @@
         </is>
       </c>
       <c r="E2" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/25 ، 2026/11/01 ، 2026/11/08 ، 2026/11/23 ، 2026/12/06 ، 2026/12/17 ، 2027/02/14 ، 2027/02/28 ، 2027/03/14 ، 2027/03/21 ، 2027/04/05 ، 2027/04/11 ، 2027/04/25 ، 2027/05/02 ، 2027/05/11 ، 2027/05/17 ، 2027/05/23</t>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/27 ، 2026/09/02 ، 2026/09/14 ، 2026/10/12 ، 2026/10/18 ، 2026/10/27 ، 2026/11/02 ، 2026/11/08 ، 2026/11/23 ، 2026/12/06 ، 2026/12/17 ، 2027/02/14 ، 2027/02/28 ، 2027/03/14 ، 2027/03/21 ، 2027/04/05 ، 2027/04/11 ، 2027/04/25 ، 2027/05/02 ، 2027/05/11 ، 2027/05/17 ، 2027/05/23</t>
         </is>
       </c>
     </row>
@@ -573,14 +582,17 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="F3" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/29 ، 2026/11/04 ، 2026/11/18 ، 2026/11/26 ، 2026/12/02 ، 2026/12/09 ، 2026/12/18 ، 2026/12/24 ، 2026/12/31 ، 2027/01/06 ، 2027/02/09 ، 2027/02/18 ، 2027/02/27 ، 2027/03/16 ، 2027/03/31 ، 2027/04/10 ، 2027/04/16 ، 2027/04/22 ، 2027/04/28 ، 2027/05/04</t>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/24 ، 2026/08/30 ، 2026/09/05 ، 2026/09/11 ، 2026/09/17 ، 2026/10/07 ، 2026/10/16 ، 2026/10/22 ، 2026/10/29 ، 2026/11/04 ، 2026/11/18 ، 2026/11/26 ، 2026/12/02 ، 2026/12/09 ، 2026/12/18 ، 2026/12/24 ، 2026/12/31 ، 2027/01/06 ، 2027/02/09 ، 2027/02/18 ، 2027/02/27 ، 2027/03/16 ، 2027/03/31 ، 2027/04/10 ، 2027/04/16 ، 2027/04/22 ، 2027/04/28 ، 2027/05/04</t>
         </is>
       </c>
     </row>
@@ -606,14 +618,17 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="F4" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/26 ، 2026/11/05 ، 2026/11/16 ، 2026/11/23 ، 2026/11/30 ، 2026/12/07 ، 2026/12/17 ، 2026/12/23 ، 2026/12/29 ، 2027/01/04 ، 2027/01/24 ، 2027/01/31 ، 2027/02/06 ، 2027/02/13 ، 2027/02/23 ، 2027/03/01 ، 2027/03/07 ، 2027/04/03 ، 2027/04/13 ، 2027/04/19</t>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>2026/10/12 ، 2026/10/19 ، 2026/10/26 ، 2026/11/05 ، 2026/11/16 ، 2026/11/23 ، 2026/11/30 ، 2026/12/07 ، 2026/12/17 ، 2026/12/23 ، 2026/12/29 ، 2027/01/04 ، 2027/01/24 ، 2027/01/31 ، 2027/02/06 ، 2027/02/13 ، 2027/02/23 ، 2027/03/01 ، 2027/03/07 ، 2027/04/03 ، 2027/04/13 ، 2027/04/19</t>
         </is>
       </c>
     </row>
@@ -644,7 +659,10 @@
       <c r="F5" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>2026/11/02 ، 2026/11/16 ، 2026/11/23 ، 2026/11/30 ، 2026/12/07 ، 2026/12/14 ، 2026/12/21 ، 2026/12/28 ، 2027/01/04 ، 2027/01/25 ، 2027/02/08 ، 2027/02/15 ، 2027/02/22 ، 2027/03/01</t>
         </is>
@@ -672,14 +690,17 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="F6" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/28 ، 2026/11/04 ، 2026/11/18 ، 2026/11/26 ، 2026/12/02 ، 2026/12/09 ، 2027/01/24 ، 2027/02/06 ، 2027/02/12 ، 2027/02/18 ، 2027/02/24 ، 2027/03/17</t>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/26 ، 2026/09/02 ، 2026/09/09 ، 2026/09/16 ، 2026/10/07 ، 2026/10/15 ، 2026/10/21 ، 2026/10/28 ، 2026/11/04 ، 2026/11/18 ، 2026/11/26 ، 2026/12/02 ، 2026/12/09 ، 2027/01/24 ، 2027/02/06 ، 2027/02/12 ، 2027/02/18 ، 2027/02/24 ، 2027/03/17</t>
         </is>
       </c>
     </row>
@@ -705,14 +726,17 @@
         </is>
       </c>
       <c r="E7" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="F7" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/03 ، 2026/12/01 ، 2026/12/15 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/23 ، 2027/03/02 ، 2027/03/31 ، 2027/04/06 ، 2027/04/20 ، 2027/04/27 ، 2027/05/09 ، 2027/05/25</t>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/08 ، 2026/10/07 ، 2026/10/13 ، 2026/10/20 ، 2026/11/03 ، 2026/12/01 ، 2026/12/15 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/23 ، 2027/03/02 ، 2027/03/31 ، 2027/04/06 ، 2027/04/20 ، 2027/04/27 ، 2027/05/09 ، 2027/05/25</t>
         </is>
       </c>
     </row>
@@ -738,14 +762,17 @@
         </is>
       </c>
       <c r="E8" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="F8" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/26 ، 2026/11/23 ، 2026/11/30 ، 2026/12/15 ، 2026/12/21 ، 2027/02/01 ، 2027/02/08 ، 2027/02/22 ، 2027/03/01 ، 2027/04/05 ، 2027/04/19 ، 2027/04/26 ، 2027/05/03 ، 2027/05/14 ، 2027/05/24</t>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/07 ، 2026/10/26 ، 2026/11/23 ، 2026/11/30 ، 2026/12/15 ، 2026/12/21 ، 2027/02/01 ، 2027/02/08 ، 2027/02/22 ، 2027/03/01 ، 2027/04/05 ، 2027/04/19 ، 2027/04/26 ، 2027/05/03 ، 2027/05/14 ، 2027/05/24</t>
         </is>
       </c>
     </row>
@@ -771,14 +798,17 @@
         </is>
       </c>
       <c r="E9" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="F9" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/27 ، 2026/11/03 ، 2026/12/01 ، 2026/12/15 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/16 ، 2027/02/23 ، 2027/03/02 ، 2027/03/31 ، 2027/04/06 ، 2027/04/13 ، 2027/04/27 ، 2027/05/13 ، 2027/05/25</t>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/08 ، 2026/10/07 ، 2026/10/13 ، 2026/10/20 ، 2026/10/27 ، 2026/11/03 ، 2026/12/01 ، 2026/12/15 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/16 ، 2027/02/23 ، 2027/03/02 ، 2027/03/31 ، 2027/04/06 ، 2027/04/13 ، 2027/04/27 ، 2027/05/13 ، 2027/05/25</t>
         </is>
       </c>
     </row>
@@ -804,14 +834,17 @@
         </is>
       </c>
       <c r="E10" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="F10" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/02 ، 2026/12/01 ، 2026/12/07 ، 2026/12/22 ، 2027/02/01 ، 2027/02/08 ، 2027/02/15 ، 2027/02/22 ، 2027/03/01 ، 2027/04/05 ، 2027/04/20 ، 2027/04/26 ، 2027/05/10 ، 2027/05/24</t>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/07 ، 2026/10/17 ، 2026/11/02 ، 2026/12/01 ، 2026/12/07 ، 2026/12/22 ، 2027/02/01 ، 2027/02/08 ، 2027/02/15 ، 2027/02/22 ، 2027/03/01 ، 2027/04/05 ، 2027/04/20 ، 2027/04/26 ، 2027/05/10 ، 2027/05/24</t>
         </is>
       </c>
     </row>
@@ -837,14 +870,17 @@
         </is>
       </c>
       <c r="E11" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="F11" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/03 ، 2026/12/01 ، 2026/12/08 ، 2026/12/15 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/16 ، 2027/02/23 ، 2027/03/02 ، 2027/04/13 ، 2027/05/04</t>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/08 ، 2026/09/15 ، 2026/10/07 ، 2026/10/13 ، 2026/10/20 ، 2026/11/03 ، 2026/12/01 ، 2026/12/08 ، 2026/12/15 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/16 ، 2027/02/23 ، 2027/03/02 ، 2027/04/13 ، 2027/05/04</t>
         </is>
       </c>
     </row>
@@ -870,14 +906,17 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="F12" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/02 ، 2026/11/30 ، 2026/12/07 ، 2026/12/14 ، 2026/12/21 ، 2027/02/01 ، 2027/02/08 ، 2027/02/15 ، 2027/02/22 ، 2027/03/01 ، 2027/03/16 ، 2027/04/05 ، 2027/04/12 ، 2027/04/19 ، 2027/05/03</t>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/07 ، 2026/09/14 ، 2026/10/12 ، 2026/10/19 ، 2026/11/02 ، 2026/11/30 ، 2026/12/07 ، 2026/12/14 ، 2026/12/21 ، 2027/02/01 ، 2027/02/08 ، 2027/02/15 ، 2027/02/22 ، 2027/03/01 ، 2027/03/16 ، 2027/04/05 ، 2027/04/12 ، 2027/04/19 ، 2027/05/03</t>
         </is>
       </c>
     </row>
@@ -903,14 +942,17 @@
         </is>
       </c>
       <c r="E13" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="F13" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/27 ، 2026/11/03 ، 2026/12/01 ، 2026/12/08 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/16 ، 2027/03/02 ، 2027/03/31 ، 2027/04/20 ، 2027/04/27 ، 2027/05/04</t>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/08 ، 2026/09/15 ، 2026/10/07 ، 2026/10/13 ، 2026/10/20 ، 2026/10/27 ، 2026/11/03 ، 2026/12/01 ، 2026/12/08 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/16 ، 2027/03/02 ، 2027/03/31 ، 2027/04/20 ، 2027/04/27 ، 2027/05/04</t>
         </is>
       </c>
     </row>
@@ -936,14 +978,17 @@
         </is>
       </c>
       <c r="E14" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="F14" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/26 ، 2026/11/02 ، 2026/12/01 ، 2026/12/07 ، 2026/12/22 ، 2027/02/01 ، 2027/02/08 ، 2027/02/15 ، 2027/03/02 ، 2027/04/13 ، 2027/04/19 ، 2027/04/26 ، 2027/05/03</t>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/07 ، 2026/09/14 ، 2026/10/12 ، 2026/10/19 ، 2026/10/26 ، 2026/11/02 ، 2026/12/01 ، 2026/12/07 ، 2026/12/22 ، 2027/02/01 ، 2027/02/08 ، 2027/02/15 ، 2027/03/02 ، 2027/04/13 ، 2027/04/19 ، 2027/04/26 ، 2027/05/03</t>
         </is>
       </c>
     </row>
@@ -965,14 +1010,17 @@
         </is>
       </c>
       <c r="E15" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="G15" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="F15" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/25 ، 2026/11/18 ، 2026/12/17 ، 2027/02/14 ، 2027/03/01 ، 2027/03/14 ، 2027/03/31 ، 2027/04/06 ، 2027/04/12 ، 2027/05/02 ، 2027/05/11 ، 2027/05/17 ، 2027/05/23</t>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/27 ، 2026/09/02 ، 2026/09/14 ، 2026/10/25 ، 2026/11/18 ، 2026/12/17 ، 2027/02/14 ، 2027/03/01 ، 2027/03/14 ، 2027/03/31 ، 2027/04/06 ، 2027/04/12 ، 2027/05/02 ، 2027/05/11 ، 2027/05/17 ، 2027/05/23</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1058,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>2) بدأ العدّ من 23/10/2026 (الغد)، لأن المباريات التي سبقت اليوم لا يمكن تأجيلها الآن.</t>
+          <t>2) بدأ العدّ من أول جولة في كل دوري (بداية الموسم). وعمود «منها مواعيد ما زالت متاحة بعد اليوم» يبيّن كم موعداً من هذه المواعيد لم يمضِ بعد، لأن الموعد الذي مضى ولم يُستخدم لا يمكن الرجوع إليه.</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1121,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>- مواعيد المؤجلات الرسمية في ورقة PRO بعد اليوم: 21/2، 7/4، 12/4، 3/5، 10-11/5، 17-18/5 من عام 2027 (6 مواعيد).</t>
+          <t>- مواعيد المؤجلات الرسمية في ورقة PRO طوال الموسم: 1/9/2026، ثم 21/2، 7/4، 12/4، 3/5، 10-11/5، 17-18/5 من عام 2027 (7 مواعيد).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Count postponement dates from today, accepting matches postponed since round 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019JaUXG9cM9tqcS3gAAknD4
</commit_message>
<xml_diff>
--- a/نتيجة_المباريات_المؤجلة_2026-27.xlsx
+++ b/نتيجة_المباريات_المؤجلة_2026-27.xlsx
@@ -505,7 +505,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>عدد المباريات التي يمكن تأجيلها (الرقم المعتمد)</t>
+          <t>عدد المواعيد المتاحة للمؤجلات من الغد 23/10/2026 حتى نهاية الموسم (الرقم المعتمد)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -515,12 +515,12 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>منها مواعيد ما زالت متاحة بعد اليوم 22/10/2026</t>
+          <t>للمقارنة: العدد لو حُسب من أول جولة في الموسم</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>التواريخ المقترحة للمباريات المؤجلة</t>
+          <t>التواريخ المقترحة (من الغد فصاعداً)</t>
         </is>
       </c>
     </row>
@@ -546,17 +546,17 @@
         </is>
       </c>
       <c r="E2" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>17</v>
-      </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>2026/08/27 ، 2026/09/02 ، 2026/09/14 ، 2026/10/12 ، 2026/10/18 ، 2026/10/27 ، 2026/11/02 ، 2026/11/08 ، 2026/11/23 ، 2026/12/06 ، 2026/12/17 ، 2027/02/14 ، 2027/02/28 ، 2027/03/14 ، 2027/03/21 ، 2027/04/05 ، 2027/04/11 ، 2027/04/25 ، 2027/05/02 ، 2027/05/11 ، 2027/05/17 ، 2027/05/23</t>
+          <t>2026/10/25 ، 2026/11/01 ، 2026/11/08 ، 2026/11/23 ، 2026/12/06 ، 2026/12/17 ، 2027/02/14 ، 2027/02/28 ، 2027/03/14 ، 2027/03/21 ، 2027/04/05 ، 2027/04/11 ، 2027/04/25 ، 2027/05/02 ، 2027/05/11 ، 2027/05/17 ، 2027/05/23</t>
         </is>
       </c>
     </row>
@@ -582,17 +582,17 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="F3" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>20</v>
-      </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>2026/08/24 ، 2026/08/30 ، 2026/09/05 ، 2026/09/11 ، 2026/09/17 ، 2026/10/07 ، 2026/10/16 ، 2026/10/22 ، 2026/10/29 ، 2026/11/04 ، 2026/11/18 ، 2026/11/26 ، 2026/12/02 ، 2026/12/09 ، 2026/12/18 ، 2026/12/24 ، 2026/12/31 ، 2027/01/06 ، 2027/02/09 ، 2027/02/18 ، 2027/02/27 ، 2027/03/16 ، 2027/03/31 ، 2027/04/10 ، 2027/04/16 ، 2027/04/22 ، 2027/04/28 ، 2027/05/04</t>
+          <t>2026/10/23 ، 2026/10/29 ، 2026/11/04 ، 2026/11/18 ، 2026/11/26 ، 2026/12/02 ، 2026/12/09 ، 2026/12/18 ، 2026/12/24 ، 2026/12/31 ، 2027/01/06 ، 2027/02/09 ، 2027/02/18 ، 2027/02/27 ، 2027/03/16 ، 2027/03/31 ، 2027/04/10 ، 2027/04/16 ، 2027/04/22 ، 2027/04/28 ، 2027/05/04</t>
         </is>
       </c>
     </row>
@@ -618,17 +618,17 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>26</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>2026/10/12 ، 2026/10/19 ، 2026/10/26 ، 2026/11/05 ، 2026/11/16 ، 2026/11/23 ، 2026/11/30 ، 2026/12/07 ، 2026/12/17 ، 2026/12/23 ، 2026/12/29 ، 2027/01/04 ، 2027/01/24 ، 2027/01/31 ، 2027/02/06 ، 2027/02/13 ، 2027/02/23 ، 2027/03/01 ، 2027/03/07 ، 2027/04/03 ، 2027/04/13 ، 2027/04/19</t>
+          <t>2026/10/26 ، 2026/11/05 ، 2026/11/16 ، 2026/11/23 ، 2026/11/30 ، 2026/12/07 ، 2026/12/17 ، 2026/12/23 ، 2026/12/29 ، 2027/01/04 ، 2027/01/24 ، 2027/01/31 ، 2027/02/06 ، 2027/02/13 ، 2027/02/23 ، 2027/03/01 ، 2027/03/07 ، 2027/04/03 ، 2027/04/13 ، 2027/04/19</t>
         </is>
       </c>
     </row>
@@ -690,17 +690,17 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>19</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>2026/08/26 ، 2026/09/02 ، 2026/09/09 ، 2026/09/16 ، 2026/10/07 ، 2026/10/15 ، 2026/10/21 ، 2026/10/28 ، 2026/11/04 ، 2026/11/18 ، 2026/11/26 ، 2026/12/02 ، 2026/12/09 ، 2027/01/24 ، 2027/02/06 ، 2027/02/12 ، 2027/02/18 ، 2027/02/24 ، 2027/03/17</t>
+          <t>2026/10/23 ، 2026/10/29 ، 2026/11/04 ، 2026/11/18 ، 2026/11/26 ، 2026/12/02 ، 2026/12/09 ، 2027/01/24 ، 2027/02/06 ، 2027/02/12 ، 2027/02/18 ، 2027/02/24 ، 2027/03/17</t>
         </is>
       </c>
     </row>
@@ -726,17 +726,17 @@
         </is>
       </c>
       <c r="E7" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="F7" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>14</v>
-      </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>2026/09/08 ، 2026/10/07 ، 2026/10/13 ، 2026/10/20 ، 2026/11/03 ، 2026/12/01 ، 2026/12/15 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/23 ، 2027/03/02 ، 2027/03/31 ، 2027/04/06 ، 2027/04/20 ، 2027/04/27 ، 2027/05/09 ، 2027/05/25</t>
+          <t>2026/11/03 ، 2026/12/01 ، 2026/12/15 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/23 ، 2027/03/02 ، 2027/03/31 ، 2027/04/06 ، 2027/04/20 ، 2027/04/27 ، 2027/05/09 ، 2027/05/25</t>
         </is>
       </c>
     </row>
@@ -762,17 +762,17 @@
         </is>
       </c>
       <c r="E8" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="F8" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>15</v>
-      </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>2026/09/07 ، 2026/10/26 ، 2026/11/23 ، 2026/11/30 ، 2026/12/15 ، 2026/12/21 ، 2027/02/01 ، 2027/02/08 ، 2027/02/22 ، 2027/03/01 ، 2027/04/05 ، 2027/04/19 ، 2027/04/26 ، 2027/05/03 ، 2027/05/14 ، 2027/05/24</t>
+          <t>2026/10/26 ، 2026/11/23 ، 2026/11/30 ، 2026/12/15 ، 2026/12/21 ، 2027/02/01 ، 2027/02/08 ، 2027/02/22 ، 2027/03/01 ، 2027/04/05 ، 2027/04/19 ، 2027/04/26 ، 2027/05/03 ، 2027/05/14 ، 2027/05/24</t>
         </is>
       </c>
     </row>
@@ -798,17 +798,17 @@
         </is>
       </c>
       <c r="E9" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="F9" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>16</v>
-      </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026/09/08 ، 2026/10/07 ، 2026/10/13 ، 2026/10/20 ، 2026/10/27 ، 2026/11/03 ، 2026/12/01 ، 2026/12/15 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/16 ، 2027/02/23 ، 2027/03/02 ، 2027/03/31 ، 2027/04/06 ، 2027/04/13 ، 2027/04/27 ، 2027/05/13 ، 2027/05/25</t>
+          <t>2026/10/27 ، 2026/11/03 ، 2026/12/01 ، 2026/12/15 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/16 ، 2027/02/23 ، 2027/03/02 ، 2027/03/31 ، 2027/04/06 ، 2027/04/13 ، 2027/04/27 ، 2027/05/13 ، 2027/05/25</t>
         </is>
       </c>
     </row>
@@ -834,17 +834,17 @@
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>29</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>2026/09/07 ، 2026/10/17 ، 2026/11/02 ، 2026/12/01 ، 2026/12/07 ، 2026/12/22 ، 2027/02/01 ، 2027/02/08 ، 2027/02/15 ، 2027/02/22 ، 2027/03/01 ، 2027/04/05 ، 2027/04/20 ، 2027/04/26 ، 2027/05/10 ، 2027/05/24</t>
+          <t>2026/10/23 ، 2026/11/02 ، 2026/12/01 ، 2026/12/07 ، 2026/12/22 ، 2027/02/01 ، 2027/02/08 ، 2027/02/15 ، 2027/02/22 ، 2027/03/01 ، 2027/04/05 ، 2027/04/20 ، 2027/04/26 ، 2027/05/10 ، 2027/05/24</t>
         </is>
       </c>
     </row>
@@ -870,17 +870,17 @@
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>25</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>2026/09/08 ، 2026/09/15 ، 2026/10/07 ، 2026/10/13 ، 2026/10/20 ، 2026/11/03 ، 2026/12/01 ، 2026/12/08 ، 2026/12/15 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/16 ، 2027/02/23 ، 2027/03/02 ، 2027/04/13 ، 2027/05/04</t>
+          <t>2026/11/03 ، 2026/12/01 ، 2026/12/08 ، 2026/12/15 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/16 ، 2027/02/23 ، 2027/03/02 ، 2027/04/13 ، 2027/05/04</t>
         </is>
       </c>
     </row>
@@ -906,17 +906,17 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>28</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>2026/09/07 ، 2026/09/14 ، 2026/10/12 ، 2026/10/19 ، 2026/11/02 ، 2026/11/30 ، 2026/12/07 ، 2026/12/14 ، 2026/12/21 ، 2027/02/01 ، 2027/02/08 ، 2027/02/15 ، 2027/02/22 ، 2027/03/01 ، 2027/03/16 ، 2027/04/05 ، 2027/04/12 ، 2027/04/19 ، 2027/05/03</t>
+          <t>2026/10/23 ، 2026/11/02 ، 2026/11/30 ، 2026/12/07 ، 2026/12/14 ، 2026/12/21 ، 2027/02/01 ، 2027/02/08 ، 2027/02/15 ، 2027/02/22 ، 2027/03/01 ، 2027/03/16 ، 2027/04/05 ، 2027/04/12 ، 2027/04/19 ، 2027/05/03</t>
         </is>
       </c>
     </row>
@@ -942,17 +942,17 @@
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>28</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>2026/09/08 ، 2026/09/15 ، 2026/10/07 ، 2026/10/13 ، 2026/10/20 ، 2026/10/27 ، 2026/11/03 ، 2026/12/01 ، 2026/12/08 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/16 ، 2027/03/02 ، 2027/03/31 ، 2027/04/20 ، 2027/04/27 ، 2027/05/04</t>
+          <t>2026/10/27 ، 2026/11/03 ، 2026/12/01 ، 2026/12/08 ، 2026/12/22 ، 2027/02/02 ، 2027/02/09 ، 2027/02/16 ، 2027/03/02 ، 2027/03/31 ، 2027/04/20 ، 2027/04/27 ، 2027/05/04</t>
         </is>
       </c>
     </row>
@@ -978,17 +978,17 @@
         </is>
       </c>
       <c r="E14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G14" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="F14" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>13</v>
-      </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026/09/07 ، 2026/09/14 ، 2026/10/12 ، 2026/10/19 ، 2026/10/26 ، 2026/11/02 ، 2026/12/01 ، 2026/12/07 ، 2026/12/22 ، 2027/02/01 ، 2027/02/08 ، 2027/02/15 ، 2027/03/02 ، 2027/04/13 ، 2027/04/19 ، 2027/04/26 ، 2027/05/03</t>
+          <t>2026/10/26 ، 2026/11/02 ، 2026/12/01 ، 2026/12/07 ، 2026/12/22 ، 2027/02/01 ، 2027/02/08 ، 2027/02/15 ، 2027/03/02 ، 2027/04/13 ، 2027/04/19 ، 2027/04/26 ، 2027/05/03</t>
         </is>
       </c>
     </row>
@@ -1010,17 +1010,17 @@
         </is>
       </c>
       <c r="E15" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="G15" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="F15" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>13</v>
-      </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>2026/08/27 ، 2026/09/02 ، 2026/09/14 ، 2026/10/25 ، 2026/11/18 ، 2026/12/17 ، 2027/02/14 ، 2027/03/01 ، 2027/03/14 ، 2027/03/31 ، 2027/04/06 ، 2027/04/12 ، 2027/05/02 ، 2027/05/11 ، 2027/05/17 ، 2027/05/23</t>
+          <t>2026/10/25 ، 2026/11/18 ، 2026/12/17 ، 2027/02/14 ، 2027/03/01 ، 2027/03/14 ، 2027/03/31 ، 2027/04/06 ، 2027/04/12 ، 2027/05/02 ، 2027/05/11 ، 2027/05/17 ، 2027/05/23</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>2) بدأ العدّ من أول جولة في كل دوري (بداية الموسم). وعمود «منها مواعيد ما زالت متاحة بعد اليوم» يبيّن كم موعداً من هذه المواعيد لم يمضِ بعد، لأن الموعد الذي مضى ولم يُستخدم لا يمكن الرجوع إليه.</t>
+          <t>2) المواعيد المحسوبة تبدأ من الغد 23/10/2026، لأن أي مباراة مؤجلة (سواء أُجّلت من الجولات الماضية أو ستؤجَّل لاحقاً) لم تُلعب بعد، ولا يمكن لعبها في يوم مضى. ويصلح الموعد لأي مباراة أُجّلت من جولة سابقة له، منذ أول جولة في الدوري.</t>
         </is>
       </c>
     </row>

</xml_diff>